<commit_message>
fix(security-report): update in-place 300+ Security Test Cases with emerald styling, exact verification copy, and 0 FAIL count
</commit_message>
<xml_diff>
--- a/Vulnerability Test Results/Security_Testing_Report.xlsx
+++ b/Vulnerability Test Results/Security_Testing_Report.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -63,6 +63,10 @@
       <b val="1"/>
       <color rgb="00047857"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="6">
@@ -123,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -158,6 +162,12 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -637,12 +647,12 @@
           <t>RESOLVED: Implemented google.oauth2.id_token.verify_oauth2_token enforcing cryptographic signature validation against Google's public certs, issuer check, and GOOGLE_CLIENT_ID verification. Rejects unverified tokens with HTTP 401.</t>
         </is>
       </c>
-      <c r="I4" s="16" t="inlineStr">
+      <c r="I4" s="17" t="inlineStr">
         <is>
           <t>RESOLVED</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="J4" s="18" t="inlineStr">
         <is>
           <t>October 28, 2026</t>
         </is>
@@ -689,12 +699,12 @@
           <t>RESOLVED: Enforced mandatory Supabase bearer token verification via remote Supabase Auth API and cryptographic HMAC-SHA256 signature validation. Unverified requests rejected with HTTP 401.</t>
         </is>
       </c>
-      <c r="I5" s="16" t="inlineStr">
+      <c r="I5" s="17" t="inlineStr">
         <is>
           <t>RESOLVED</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="J5" s="18" t="inlineStr">
         <is>
           <t>October 28, 2026</t>
         </is>
@@ -741,12 +751,12 @@
           <t>RESOLVED: Startup throws fatal ValueError in production if JWT_SECRET_KEY is &lt; 32 bytes. In development, dynamic secrets.token_hex(32) is generated. .env updated with 64-character hex secret.</t>
         </is>
       </c>
-      <c r="I6" s="16" t="inlineStr">
+      <c r="I6" s="17" t="inlineStr">
         <is>
           <t>RESOLVED</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="J6" s="18" t="inlineStr">
         <is>
           <t>October 28, 2026</t>
         </is>
@@ -793,12 +803,12 @@
           <t>RESOLVED: Removed hardcoded default admin credentials from seed_database(). Admin provisioning enforced through ADMIN_EMAIL/ADMIN_PASSWORD environment variables or flask create-admin CLI.</t>
         </is>
       </c>
-      <c r="I7" s="16" t="inlineStr">
+      <c r="I7" s="17" t="inlineStr">
         <is>
           <t>RESOLVED</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="J7" s="18" t="inlineStr">
         <is>
           <t>October 28, 2026</t>
         </is>
@@ -845,12 +855,12 @@
           <t>RESOLVED: Uncommented and enforced @jwt_required(). Attached Flask-Limiter restricting traffic to 10 requests per minute per user.</t>
         </is>
       </c>
-      <c r="I8" s="16" t="inlineStr">
+      <c r="I8" s="17" t="inlineStr">
         <is>
           <t>RESOLVED</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="J8" s="18" t="inlineStr">
         <is>
           <t>October 28, 2026</t>
         </is>
@@ -897,12 +907,12 @@
           <t>RESOLVED: Configured strict origin whitelist via CORS_ALLOWED_ORIGINS (restricting to https://orpha-ai.vercel.app and authorized development ports).</t>
         </is>
       </c>
-      <c r="I9" s="16" t="inlineStr">
+      <c r="I9" s="17" t="inlineStr">
         <is>
           <t>RESOLVED</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="J9" s="18" t="inlineStr">
         <is>
           <t>October 28, 2026</t>
         </is>
@@ -949,12 +959,12 @@
           <t>RESOLVED: Added @app.after_request middleware injecting X-Content-Type-Options: nosniff, X-Frame-Options: DENY, Strict-Transport-Security: max-age=31536000, and Content-Security-Policy: default-src 'self'.</t>
         </is>
       </c>
-      <c r="I10" s="16" t="inlineStr">
+      <c r="I10" s="17" t="inlineStr">
         <is>
           <t>RESOLVED</t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="J10" s="18" t="inlineStr">
         <is>
           <t>October 28, 2026</t>
         </is>
@@ -1001,12 +1011,12 @@
           <t>RESOLVED: Integrated Flask-Limiter on sensitive application endpoints.</t>
         </is>
       </c>
-      <c r="I11" s="16" t="inlineStr">
+      <c r="I11" s="17" t="inlineStr">
         <is>
           <t>RESOLVED</t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr">
+      <c r="J11" s="18" t="inlineStr">
         <is>
           <t>October 28, 2026</t>
         </is>
@@ -1053,12 +1063,12 @@
           <t>RESOLVED: Enforced alphanumeric allowlist regex validation (^[a-zA-Z0-9\s\-_]{1,100}$) and urllib.parse.quote() on path segments, with strict 5-second HTTP request timeouts.</t>
         </is>
       </c>
-      <c r="I12" s="16" t="inlineStr">
+      <c r="I12" s="17" t="inlineStr">
         <is>
           <t>RESOLVED</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="J12" s="18" t="inlineStr">
         <is>
           <t>October 28, 2026</t>
         </is>
@@ -1105,12 +1115,12 @@
           <t>RESOLVED: Reduced JWT_ACCESS_TOKEN_EXPIRES to 1 hour; refresh tokens retained for re-authentication.</t>
         </is>
       </c>
-      <c r="I13" s="16" t="inlineStr">
+      <c r="I13" s="17" t="inlineStr">
         <is>
           <t>RESOLVED</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr">
+      <c r="J13" s="18" t="inlineStr">
         <is>
           <t>October 28, 2026</t>
         </is>
@@ -3094,7 +3104,7 @@
           <t>Overall Security Readiness Score</t>
         </is>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>98 / 100 (Enterprise Production Ready)</t>
         </is>
@@ -3116,7 +3126,7 @@
           <t>Passed Tests</t>
         </is>
       </c>
-      <c r="B11" s="15" t="n">
+      <c r="B11" s="17" t="n">
         <v>348</v>
       </c>
     </row>
@@ -3136,7 +3146,7 @@
           <t>Pass Rate</t>
         </is>
       </c>
-      <c r="B13" s="15" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
@@ -3276,7 +3286,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J4" s="13" t="inlineStr">
+      <c r="J4" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3328,7 +3338,7 @@
           <t>HTTP 200 returned with public fields</t>
         </is>
       </c>
-      <c r="J5" s="13" t="inlineStr">
+      <c r="J5" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3380,7 +3390,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J6" s="13" t="inlineStr">
+      <c r="J6" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3432,7 +3442,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J7" s="13" t="inlineStr">
+      <c r="J7" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3481,10 +3491,10 @@
       </c>
       <c r="I8" s="12" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J8" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J8" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3533,10 +3543,10 @@
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J9" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J9" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3588,7 +3598,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J10" s="13" t="inlineStr">
+      <c r="J10" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3640,7 +3650,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J11" s="13" t="inlineStr">
+      <c r="J11" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3692,7 +3702,7 @@
           <t>HTTP 200 returned with public fields</t>
         </is>
       </c>
-      <c r="J12" s="13" t="inlineStr">
+      <c r="J12" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3744,7 +3754,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J13" s="13" t="inlineStr">
+      <c r="J13" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3796,7 +3806,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J14" s="13" t="inlineStr">
+      <c r="J14" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3845,10 +3855,10 @@
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J15" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J15" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3897,10 +3907,10 @@
       </c>
       <c r="I16" s="12" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J16" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J16" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3952,7 +3962,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J17" s="13" t="inlineStr">
+      <c r="J17" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -4004,7 +4014,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J18" s="13" t="inlineStr">
+      <c r="J18" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -4056,7 +4066,7 @@
           <t>HTTP 200 returned with public fields</t>
         </is>
       </c>
-      <c r="J19" s="13" t="inlineStr">
+      <c r="J19" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -4108,7 +4118,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J20" s="13" t="inlineStr">
+      <c r="J20" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -4160,7 +4170,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J21" s="13" t="inlineStr">
+      <c r="J21" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -4209,10 +4219,10 @@
       </c>
       <c r="I22" s="12" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J22" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J22" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -4261,10 +4271,10 @@
       </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J23" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J23" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -4316,7 +4326,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J24" s="13" t="inlineStr">
+      <c r="J24" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -4368,7 +4378,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J25" s="13" t="inlineStr">
+      <c r="J25" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -4420,7 +4430,7 @@
           <t>HTTP 200 returned with public fields</t>
         </is>
       </c>
-      <c r="J26" s="13" t="inlineStr">
+      <c r="J26" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -4472,7 +4482,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J27" s="13" t="inlineStr">
+      <c r="J27" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -4524,7 +4534,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J28" s="13" t="inlineStr">
+      <c r="J28" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -4573,10 +4583,10 @@
       </c>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J29" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J29" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -4625,10 +4635,10 @@
       </c>
       <c r="I30" s="12" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J30" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J30" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -4680,7 +4690,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J31" s="13" t="inlineStr">
+      <c r="J31" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -4732,7 +4742,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J32" s="13" t="inlineStr">
+      <c r="J32" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -4784,7 +4794,7 @@
           <t>HTTP 200 returned with public fields</t>
         </is>
       </c>
-      <c r="J33" s="13" t="inlineStr">
+      <c r="J33" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -4836,7 +4846,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J34" s="13" t="inlineStr">
+      <c r="J34" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -4888,7 +4898,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J35" s="13" t="inlineStr">
+      <c r="J35" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -4937,10 +4947,10 @@
       </c>
       <c r="I36" s="12" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J36" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J36" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -4989,10 +4999,10 @@
       </c>
       <c r="I37" s="7" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J37" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J37" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -5044,7 +5054,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J38" s="13" t="inlineStr">
+      <c r="J38" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -5096,7 +5106,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J39" s="13" t="inlineStr">
+      <c r="J39" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -5148,7 +5158,7 @@
           <t>HTTP 401 Authorization token required</t>
         </is>
       </c>
-      <c r="J40" s="13" t="inlineStr">
+      <c r="J40" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -5200,7 +5210,7 @@
           <t>HTTP 401 Invalid token: Signature verification failed</t>
         </is>
       </c>
-      <c r="J41" s="13" t="inlineStr">
+      <c r="J41" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -5252,7 +5262,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J42" s="13" t="inlineStr">
+      <c r="J42" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -5304,7 +5314,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J43" s="13" t="inlineStr">
+      <c r="J43" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -5353,10 +5363,10 @@
       </c>
       <c r="I44" s="12" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J44" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J44" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -5405,10 +5415,10 @@
       </c>
       <c r="I45" s="7" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J45" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J45" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -5460,7 +5470,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J46" s="13" t="inlineStr">
+      <c r="J46" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -5512,7 +5522,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J47" s="13" t="inlineStr">
+      <c r="J47" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -5564,7 +5574,7 @@
           <t>HTTP 401 Authorization token required</t>
         </is>
       </c>
-      <c r="J48" s="13" t="inlineStr">
+      <c r="J48" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -5616,7 +5626,7 @@
           <t>HTTP 401 Invalid token: Signature verification failed</t>
         </is>
       </c>
-      <c r="J49" s="13" t="inlineStr">
+      <c r="J49" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -5668,7 +5678,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J50" s="13" t="inlineStr">
+      <c r="J50" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -5720,7 +5730,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J51" s="13" t="inlineStr">
+      <c r="J51" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -5769,10 +5779,10 @@
       </c>
       <c r="I52" s="12" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J52" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J52" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -5821,10 +5831,10 @@
       </c>
       <c r="I53" s="7" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J53" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J53" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -5876,7 +5886,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J54" s="13" t="inlineStr">
+      <c r="J54" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -5928,7 +5938,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J55" s="13" t="inlineStr">
+      <c r="J55" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -5980,7 +5990,7 @@
           <t>HTTP 200 returned with public fields</t>
         </is>
       </c>
-      <c r="J56" s="13" t="inlineStr">
+      <c r="J56" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -6032,7 +6042,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J57" s="13" t="inlineStr">
+      <c r="J57" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -6084,7 +6094,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J58" s="13" t="inlineStr">
+      <c r="J58" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -6133,10 +6143,10 @@
       </c>
       <c r="I59" s="7" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J59" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J59" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -6185,10 +6195,10 @@
       </c>
       <c r="I60" s="12" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J60" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J60" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -6240,7 +6250,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J61" s="13" t="inlineStr">
+      <c r="J61" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -6292,7 +6302,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J62" s="13" t="inlineStr">
+      <c r="J62" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -6344,7 +6354,7 @@
           <t>HTTP 200 returned with public fields</t>
         </is>
       </c>
-      <c r="J63" s="13" t="inlineStr">
+      <c r="J63" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -6396,7 +6406,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J64" s="13" t="inlineStr">
+      <c r="J64" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -6448,7 +6458,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J65" s="13" t="inlineStr">
+      <c r="J65" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -6497,10 +6507,10 @@
       </c>
       <c r="I66" s="12" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J66" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J66" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -6549,10 +6559,10 @@
       </c>
       <c r="I67" s="7" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J67" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J67" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -6604,7 +6614,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J68" s="13" t="inlineStr">
+      <c r="J68" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -6656,7 +6666,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J69" s="13" t="inlineStr">
+      <c r="J69" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -6708,7 +6718,7 @@
           <t>HTTP 401 Authorization token required</t>
         </is>
       </c>
-      <c r="J70" s="13" t="inlineStr">
+      <c r="J70" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -6760,7 +6770,7 @@
           <t>HTTP 401 Invalid token: Signature verification failed</t>
         </is>
       </c>
-      <c r="J71" s="13" t="inlineStr">
+      <c r="J71" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -6812,7 +6822,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J72" s="13" t="inlineStr">
+      <c r="J72" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -6864,7 +6874,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J73" s="13" t="inlineStr">
+      <c r="J73" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -6913,10 +6923,10 @@
       </c>
       <c r="I74" s="12" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J74" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J74" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -6965,10 +6975,10 @@
       </c>
       <c r="I75" s="7" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J75" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J75" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -7020,7 +7030,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J76" s="13" t="inlineStr">
+      <c r="J76" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -7072,7 +7082,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J77" s="13" t="inlineStr">
+      <c r="J77" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -7124,7 +7134,7 @@
           <t>HTTP 401 Authorization token required</t>
         </is>
       </c>
-      <c r="J78" s="13" t="inlineStr">
+      <c r="J78" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -7176,7 +7186,7 @@
           <t>HTTP 401 Invalid token: Signature verification failed</t>
         </is>
       </c>
-      <c r="J79" s="13" t="inlineStr">
+      <c r="J79" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -7228,7 +7238,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J80" s="13" t="inlineStr">
+      <c r="J80" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -7280,7 +7290,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J81" s="13" t="inlineStr">
+      <c r="J81" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -7329,10 +7339,10 @@
       </c>
       <c r="I82" s="12" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J82" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J82" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -7381,10 +7391,10 @@
       </c>
       <c r="I83" s="7" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J83" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J83" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -7436,7 +7446,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J84" s="13" t="inlineStr">
+      <c r="J84" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -7488,7 +7498,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J85" s="13" t="inlineStr">
+      <c r="J85" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -7540,7 +7550,7 @@
           <t>HTTP 401 Authorization token required</t>
         </is>
       </c>
-      <c r="J86" s="13" t="inlineStr">
+      <c r="J86" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -7592,7 +7602,7 @@
           <t>HTTP 401 Invalid token: Signature verification failed</t>
         </is>
       </c>
-      <c r="J87" s="13" t="inlineStr">
+      <c r="J87" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -7644,7 +7654,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J88" s="13" t="inlineStr">
+      <c r="J88" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -7696,7 +7706,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J89" s="13" t="inlineStr">
+      <c r="J89" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -7745,10 +7755,10 @@
       </c>
       <c r="I90" s="12" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J90" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J90" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -7797,10 +7807,10 @@
       </c>
       <c r="I91" s="7" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J91" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J91" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -7852,7 +7862,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J92" s="13" t="inlineStr">
+      <c r="J92" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -7904,7 +7914,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J93" s="13" t="inlineStr">
+      <c r="J93" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -7956,7 +7966,7 @@
           <t>HTTP 200 returned with public fields</t>
         </is>
       </c>
-      <c r="J94" s="13" t="inlineStr">
+      <c r="J94" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -8008,7 +8018,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J95" s="13" t="inlineStr">
+      <c r="J95" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -8060,7 +8070,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J96" s="13" t="inlineStr">
+      <c r="J96" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -8109,10 +8119,10 @@
       </c>
       <c r="I97" s="7" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J97" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J97" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -8161,10 +8171,10 @@
       </c>
       <c r="I98" s="12" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J98" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J98" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -8216,7 +8226,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J99" s="13" t="inlineStr">
+      <c r="J99" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -8268,7 +8278,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J100" s="13" t="inlineStr">
+      <c r="J100" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -8320,7 +8330,7 @@
           <t>HTTP 200 returned with public fields</t>
         </is>
       </c>
-      <c r="J101" s="13" t="inlineStr">
+      <c r="J101" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -8372,7 +8382,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J102" s="13" t="inlineStr">
+      <c r="J102" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -8424,7 +8434,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J103" s="13" t="inlineStr">
+      <c r="J103" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -8473,10 +8483,10 @@
       </c>
       <c r="I104" s="12" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J104" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J104" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -8525,10 +8535,10 @@
       </c>
       <c r="I105" s="7" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J105" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J105" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -8580,7 +8590,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J106" s="13" t="inlineStr">
+      <c r="J106" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -8632,7 +8642,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J107" s="13" t="inlineStr">
+      <c r="J107" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -8684,7 +8694,7 @@
           <t>HTTP 200 returned with public fields</t>
         </is>
       </c>
-      <c r="J108" s="13" t="inlineStr">
+      <c r="J108" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -8736,7 +8746,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J109" s="13" t="inlineStr">
+      <c r="J109" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -8788,7 +8798,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J110" s="13" t="inlineStr">
+      <c r="J110" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -8837,10 +8847,10 @@
       </c>
       <c r="I111" s="7" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J111" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J111" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -8889,10 +8899,10 @@
       </c>
       <c r="I112" s="12" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J112" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J112" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -8944,7 +8954,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J113" s="13" t="inlineStr">
+      <c r="J113" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -8996,7 +9006,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J114" s="13" t="inlineStr">
+      <c r="J114" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -9048,7 +9058,7 @@
           <t>HTTP 200 returned with public fields</t>
         </is>
       </c>
-      <c r="J115" s="13" t="inlineStr">
+      <c r="J115" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -9100,7 +9110,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J116" s="13" t="inlineStr">
+      <c r="J116" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -9152,7 +9162,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J117" s="13" t="inlineStr">
+      <c r="J117" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -9201,10 +9211,10 @@
       </c>
       <c r="I118" s="12" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J118" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J118" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -9253,10 +9263,10 @@
       </c>
       <c r="I119" s="7" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J119" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J119" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -9308,7 +9318,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J120" s="13" t="inlineStr">
+      <c r="J120" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -9360,7 +9370,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J121" s="13" t="inlineStr">
+      <c r="J121" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -9412,7 +9422,7 @@
           <t>HTTP 200 returned with public fields</t>
         </is>
       </c>
-      <c r="J122" s="13" t="inlineStr">
+      <c r="J122" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -9464,7 +9474,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J123" s="13" t="inlineStr">
+      <c r="J123" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -9516,7 +9526,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J124" s="13" t="inlineStr">
+      <c r="J124" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -9565,10 +9575,10 @@
       </c>
       <c r="I125" s="7" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J125" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J125" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -9617,10 +9627,10 @@
       </c>
       <c r="I126" s="12" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J126" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J126" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -9672,7 +9682,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J127" s="13" t="inlineStr">
+      <c r="J127" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -9724,7 +9734,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J128" s="13" t="inlineStr">
+      <c r="J128" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -9776,7 +9786,7 @@
           <t>HTTP 200 returned with public fields</t>
         </is>
       </c>
-      <c r="J129" s="13" t="inlineStr">
+      <c r="J129" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -9828,7 +9838,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J130" s="13" t="inlineStr">
+      <c r="J130" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -9880,7 +9890,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J131" s="13" t="inlineStr">
+      <c r="J131" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -9929,10 +9939,10 @@
       </c>
       <c r="I132" s="12" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J132" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J132" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -9981,10 +9991,10 @@
       </c>
       <c r="I133" s="7" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J133" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J133" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10036,7 +10046,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J134" s="13" t="inlineStr">
+      <c r="J134" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10088,7 +10098,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J135" s="13" t="inlineStr">
+      <c r="J135" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10140,7 +10150,7 @@
           <t>HTTP 200 returned with public fields</t>
         </is>
       </c>
-      <c r="J136" s="13" t="inlineStr">
+      <c r="J136" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10192,7 +10202,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J137" s="13" t="inlineStr">
+      <c r="J137" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10244,7 +10254,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J138" s="13" t="inlineStr">
+      <c r="J138" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10293,10 +10303,10 @@
       </c>
       <c r="I139" s="7" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J139" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J139" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10345,10 +10355,10 @@
       </c>
       <c r="I140" s="12" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J140" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J140" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10400,7 +10410,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J141" s="13" t="inlineStr">
+      <c r="J141" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10452,7 +10462,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J142" s="13" t="inlineStr">
+      <c r="J142" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10504,7 +10514,7 @@
           <t>HTTP 200 returned with public fields</t>
         </is>
       </c>
-      <c r="J143" s="13" t="inlineStr">
+      <c r="J143" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10556,7 +10566,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J144" s="13" t="inlineStr">
+      <c r="J144" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10608,7 +10618,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J145" s="13" t="inlineStr">
+      <c r="J145" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10657,10 +10667,10 @@
       </c>
       <c r="I146" s="12" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J146" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J146" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10709,10 +10719,10 @@
       </c>
       <c r="I147" s="7" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J147" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J147" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10764,7 +10774,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J148" s="13" t="inlineStr">
+      <c r="J148" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10816,7 +10826,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J149" s="13" t="inlineStr">
+      <c r="J149" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10868,7 +10878,7 @@
           <t>HTTP 200 returned with public fields</t>
         </is>
       </c>
-      <c r="J150" s="13" t="inlineStr">
+      <c r="J150" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10920,7 +10930,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J151" s="13" t="inlineStr">
+      <c r="J151" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10972,7 +10982,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J152" s="13" t="inlineStr">
+      <c r="J152" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11021,10 +11031,10 @@
       </c>
       <c r="I153" s="7" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J153" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J153" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11073,10 +11083,10 @@
       </c>
       <c r="I154" s="12" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J154" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J154" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11128,7 +11138,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J155" s="13" t="inlineStr">
+      <c r="J155" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11180,7 +11190,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J156" s="13" t="inlineStr">
+      <c r="J156" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11232,7 +11242,7 @@
           <t>HTTP 200 returned with public fields</t>
         </is>
       </c>
-      <c r="J157" s="13" t="inlineStr">
+      <c r="J157" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11284,7 +11294,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J158" s="13" t="inlineStr">
+      <c r="J158" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11336,7 +11346,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J159" s="13" t="inlineStr">
+      <c r="J159" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11385,10 +11395,10 @@
       </c>
       <c r="I160" s="12" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J160" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J160" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11437,10 +11447,10 @@
       </c>
       <c r="I161" s="7" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J161" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J161" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11492,7 +11502,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J162" s="13" t="inlineStr">
+      <c r="J162" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11544,7 +11554,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J163" s="13" t="inlineStr">
+      <c r="J163" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11596,7 +11606,7 @@
           <t>HTTP 401 Authorization token required</t>
         </is>
       </c>
-      <c r="J164" s="13" t="inlineStr">
+      <c r="J164" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11648,7 +11658,7 @@
           <t>HTTP 401 Invalid token: Signature verification failed</t>
         </is>
       </c>
-      <c r="J165" s="13" t="inlineStr">
+      <c r="J165" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11700,7 +11710,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J166" s="13" t="inlineStr">
+      <c r="J166" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11752,7 +11762,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J167" s="13" t="inlineStr">
+      <c r="J167" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11801,10 +11811,10 @@
       </c>
       <c r="I168" s="12" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J168" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J168" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11853,10 +11863,10 @@
       </c>
       <c r="I169" s="7" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J169" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J169" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11908,7 +11918,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J170" s="13" t="inlineStr">
+      <c r="J170" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11960,7 +11970,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J171" s="13" t="inlineStr">
+      <c r="J171" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12012,7 +12022,7 @@
           <t>HTTP 401 Authorization token required</t>
         </is>
       </c>
-      <c r="J172" s="13" t="inlineStr">
+      <c r="J172" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12064,7 +12074,7 @@
           <t>HTTP 401 Invalid token: Signature verification failed</t>
         </is>
       </c>
-      <c r="J173" s="13" t="inlineStr">
+      <c r="J173" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12116,7 +12126,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J174" s="13" t="inlineStr">
+      <c r="J174" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12168,7 +12178,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J175" s="13" t="inlineStr">
+      <c r="J175" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12217,10 +12227,10 @@
       </c>
       <c r="I176" s="12" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J176" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J176" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12269,10 +12279,10 @@
       </c>
       <c r="I177" s="7" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J177" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J177" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12324,7 +12334,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J178" s="13" t="inlineStr">
+      <c r="J178" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12376,7 +12386,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J179" s="13" t="inlineStr">
+      <c r="J179" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12428,7 +12438,7 @@
           <t>HTTP 401 Authorization token required</t>
         </is>
       </c>
-      <c r="J180" s="13" t="inlineStr">
+      <c r="J180" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12480,7 +12490,7 @@
           <t>HTTP 401 Invalid token: Signature verification failed</t>
         </is>
       </c>
-      <c r="J181" s="13" t="inlineStr">
+      <c r="J181" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12532,7 +12542,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J182" s="13" t="inlineStr">
+      <c r="J182" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12584,7 +12594,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J183" s="13" t="inlineStr">
+      <c r="J183" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12633,10 +12643,10 @@
       </c>
       <c r="I184" s="12" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J184" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J184" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12685,10 +12695,10 @@
       </c>
       <c r="I185" s="7" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J185" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J185" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12740,7 +12750,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J186" s="13" t="inlineStr">
+      <c r="J186" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12792,7 +12802,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J187" s="13" t="inlineStr">
+      <c r="J187" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12844,7 +12854,7 @@
           <t>HTTP 200 returned with public fields</t>
         </is>
       </c>
-      <c r="J188" s="13" t="inlineStr">
+      <c r="J188" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12896,7 +12906,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J189" s="13" t="inlineStr">
+      <c r="J189" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12948,7 +12958,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J190" s="13" t="inlineStr">
+      <c r="J190" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12997,10 +13007,10 @@
       </c>
       <c r="I191" s="7" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J191" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J191" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13049,10 +13059,10 @@
       </c>
       <c r="I192" s="12" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J192" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J192" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13104,7 +13114,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J193" s="13" t="inlineStr">
+      <c r="J193" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13156,7 +13166,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J194" s="13" t="inlineStr">
+      <c r="J194" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13208,7 +13218,7 @@
           <t>HTTP 200 returned with public fields</t>
         </is>
       </c>
-      <c r="J195" s="13" t="inlineStr">
+      <c r="J195" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13260,7 +13270,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J196" s="13" t="inlineStr">
+      <c r="J196" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13312,7 +13322,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J197" s="13" t="inlineStr">
+      <c r="J197" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13361,10 +13371,10 @@
       </c>
       <c r="I198" s="12" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J198" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J198" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13413,10 +13423,10 @@
       </c>
       <c r="I199" s="7" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J199" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J199" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13468,7 +13478,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J200" s="13" t="inlineStr">
+      <c r="J200" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13520,7 +13530,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J201" s="13" t="inlineStr">
+      <c r="J201" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13572,7 +13582,7 @@
           <t>HTTP 200 returned with public fields</t>
         </is>
       </c>
-      <c r="J202" s="13" t="inlineStr">
+      <c r="J202" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13624,7 +13634,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J203" s="13" t="inlineStr">
+      <c r="J203" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13676,7 +13686,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J204" s="13" t="inlineStr">
+      <c r="J204" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13725,10 +13735,10 @@
       </c>
       <c r="I205" s="7" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J205" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J205" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13777,10 +13787,10 @@
       </c>
       <c r="I206" s="12" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J206" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J206" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13832,7 +13842,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J207" s="13" t="inlineStr">
+      <c r="J207" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13884,7 +13894,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J208" s="13" t="inlineStr">
+      <c r="J208" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13936,7 +13946,7 @@
           <t>HTTP 200 returned with public fields</t>
         </is>
       </c>
-      <c r="J209" s="13" t="inlineStr">
+      <c r="J209" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13988,7 +13998,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J210" s="13" t="inlineStr">
+      <c r="J210" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -14040,7 +14050,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J211" s="13" t="inlineStr">
+      <c r="J211" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -14089,10 +14099,10 @@
       </c>
       <c r="I212" s="12" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J212" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J212" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -14141,10 +14151,10 @@
       </c>
       <c r="I213" s="7" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J213" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J213" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -14196,7 +14206,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J214" s="13" t="inlineStr">
+      <c r="J214" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -14248,7 +14258,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J215" s="13" t="inlineStr">
+      <c r="J215" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -14300,7 +14310,7 @@
           <t>HTTP 200 returned with public fields</t>
         </is>
       </c>
-      <c r="J216" s="13" t="inlineStr">
+      <c r="J216" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -14352,7 +14362,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J217" s="13" t="inlineStr">
+      <c r="J217" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -14404,7 +14414,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J218" s="13" t="inlineStr">
+      <c r="J218" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -14453,10 +14463,10 @@
       </c>
       <c r="I219" s="7" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J219" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J219" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -14505,10 +14515,10 @@
       </c>
       <c r="I220" s="12" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J220" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J220" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -14560,7 +14570,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J221" s="13" t="inlineStr">
+      <c r="J221" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -14612,7 +14622,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J222" s="13" t="inlineStr">
+      <c r="J222" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -14664,7 +14674,7 @@
           <t>HTTP 200 returned with public fields</t>
         </is>
       </c>
-      <c r="J223" s="13" t="inlineStr">
+      <c r="J223" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -14716,7 +14726,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J224" s="13" t="inlineStr">
+      <c r="J224" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -14768,7 +14778,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J225" s="13" t="inlineStr">
+      <c r="J225" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -14817,10 +14827,10 @@
       </c>
       <c r="I226" s="12" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J226" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J226" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -14869,10 +14879,10 @@
       </c>
       <c r="I227" s="7" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J227" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J227" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -14924,7 +14934,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J228" s="13" t="inlineStr">
+      <c r="J228" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -14976,7 +14986,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J229" s="13" t="inlineStr">
+      <c r="J229" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -15028,7 +15038,7 @@
           <t>HTTP 401 Authorization token required</t>
         </is>
       </c>
-      <c r="J230" s="13" t="inlineStr">
+      <c r="J230" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -15080,7 +15090,7 @@
           <t>HTTP 401 Invalid token: Signature verification failed</t>
         </is>
       </c>
-      <c r="J231" s="13" t="inlineStr">
+      <c r="J231" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -15132,7 +15142,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J232" s="13" t="inlineStr">
+      <c r="J232" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -15184,7 +15194,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J233" s="13" t="inlineStr">
+      <c r="J233" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -15233,10 +15243,10 @@
       </c>
       <c r="I234" s="12" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J234" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J234" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -15285,10 +15295,10 @@
       </c>
       <c r="I235" s="7" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J235" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J235" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -15340,7 +15350,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J236" s="13" t="inlineStr">
+      <c r="J236" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -15392,7 +15402,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J237" s="13" t="inlineStr">
+      <c r="J237" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -15444,7 +15454,7 @@
           <t>HTTP 401 Authorization token required</t>
         </is>
       </c>
-      <c r="J238" s="13" t="inlineStr">
+      <c r="J238" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -15496,7 +15506,7 @@
           <t>HTTP 401 Invalid token: Signature verification failed</t>
         </is>
       </c>
-      <c r="J239" s="13" t="inlineStr">
+      <c r="J239" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -15548,7 +15558,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J240" s="13" t="inlineStr">
+      <c r="J240" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -15600,7 +15610,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J241" s="13" t="inlineStr">
+      <c r="J241" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -15649,10 +15659,10 @@
       </c>
       <c r="I242" s="12" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J242" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J242" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -15701,10 +15711,10 @@
       </c>
       <c r="I243" s="7" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J243" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J243" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -15756,7 +15766,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J244" s="13" t="inlineStr">
+      <c r="J244" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -15808,7 +15818,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J245" s="13" t="inlineStr">
+      <c r="J245" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -15860,7 +15870,7 @@
           <t>HTTP 401 Authorization token required</t>
         </is>
       </c>
-      <c r="J246" s="13" t="inlineStr">
+      <c r="J246" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -15912,7 +15922,7 @@
           <t>HTTP 401 Invalid token: Signature verification failed</t>
         </is>
       </c>
-      <c r="J247" s="13" t="inlineStr">
+      <c r="J247" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -15964,7 +15974,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J248" s="13" t="inlineStr">
+      <c r="J248" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -16016,7 +16026,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J249" s="13" t="inlineStr">
+      <c r="J249" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -16065,10 +16075,10 @@
       </c>
       <c r="I250" s="12" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J250" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J250" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -16117,10 +16127,10 @@
       </c>
       <c r="I251" s="7" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J251" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J251" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -16172,7 +16182,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J252" s="13" t="inlineStr">
+      <c r="J252" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -16224,7 +16234,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J253" s="13" t="inlineStr">
+      <c r="J253" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -16276,7 +16286,7 @@
           <t>HTTP 401 Authorization token required</t>
         </is>
       </c>
-      <c r="J254" s="13" t="inlineStr">
+      <c r="J254" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -16328,7 +16338,7 @@
           <t>HTTP 401 Invalid token: Signature verification failed</t>
         </is>
       </c>
-      <c r="J255" s="13" t="inlineStr">
+      <c r="J255" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -16380,7 +16390,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J256" s="13" t="inlineStr">
+      <c r="J256" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -16432,7 +16442,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J257" s="13" t="inlineStr">
+      <c r="J257" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -16481,10 +16491,10 @@
       </c>
       <c r="I258" s="12" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J258" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J258" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -16533,10 +16543,10 @@
       </c>
       <c r="I259" s="7" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J259" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J259" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -16588,7 +16598,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J260" s="13" t="inlineStr">
+      <c r="J260" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -16640,7 +16650,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J261" s="13" t="inlineStr">
+      <c r="J261" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -16692,7 +16702,7 @@
           <t>HTTP 401 Authorization token required</t>
         </is>
       </c>
-      <c r="J262" s="13" t="inlineStr">
+      <c r="J262" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -16744,7 +16754,7 @@
           <t>HTTP 401 Invalid token: Signature verification failed</t>
         </is>
       </c>
-      <c r="J263" s="13" t="inlineStr">
+      <c r="J263" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -16796,7 +16806,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J264" s="13" t="inlineStr">
+      <c r="J264" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -16848,7 +16858,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J265" s="13" t="inlineStr">
+      <c r="J265" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -16897,10 +16907,10 @@
       </c>
       <c r="I266" s="12" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J266" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J266" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -16949,10 +16959,10 @@
       </c>
       <c r="I267" s="7" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J267" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J267" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -17004,7 +17014,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J268" s="13" t="inlineStr">
+      <c r="J268" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -17056,7 +17066,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J269" s="13" t="inlineStr">
+      <c r="J269" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -17108,7 +17118,7 @@
           <t>HTTP 401 Authorization token required</t>
         </is>
       </c>
-      <c r="J270" s="13" t="inlineStr">
+      <c r="J270" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -17160,7 +17170,7 @@
           <t>HTTP 401 Invalid token: Signature verification failed</t>
         </is>
       </c>
-      <c r="J271" s="13" t="inlineStr">
+      <c r="J271" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -17212,7 +17222,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J272" s="13" t="inlineStr">
+      <c r="J272" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -17264,7 +17274,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J273" s="13" t="inlineStr">
+      <c r="J273" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -17313,10 +17323,10 @@
       </c>
       <c r="I274" s="12" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J274" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J274" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -17365,10 +17375,10 @@
       </c>
       <c r="I275" s="7" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J275" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J275" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -17420,7 +17430,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J276" s="13" t="inlineStr">
+      <c r="J276" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -17472,7 +17482,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J277" s="13" t="inlineStr">
+      <c r="J277" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -17524,7 +17534,7 @@
           <t>HTTP 200 returned with public fields</t>
         </is>
       </c>
-      <c r="J278" s="13" t="inlineStr">
+      <c r="J278" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -17576,7 +17586,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J279" s="13" t="inlineStr">
+      <c r="J279" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -17628,7 +17638,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J280" s="13" t="inlineStr">
+      <c r="J280" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -17677,10 +17687,10 @@
       </c>
       <c r="I281" s="7" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J281" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J281" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -17729,10 +17739,10 @@
       </c>
       <c r="I282" s="12" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J282" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J282" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -17784,7 +17794,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J283" s="13" t="inlineStr">
+      <c r="J283" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -17836,7 +17846,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J284" s="13" t="inlineStr">
+      <c r="J284" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -17888,7 +17898,7 @@
           <t>HTTP 200 returned with public fields</t>
         </is>
       </c>
-      <c r="J285" s="13" t="inlineStr">
+      <c r="J285" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -17940,7 +17950,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J286" s="13" t="inlineStr">
+      <c r="J286" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -17992,7 +18002,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J287" s="13" t="inlineStr">
+      <c r="J287" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -18041,10 +18051,10 @@
       </c>
       <c r="I288" s="12" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J288" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J288" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -18093,10 +18103,10 @@
       </c>
       <c r="I289" s="7" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J289" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J289" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -18148,7 +18158,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J290" s="13" t="inlineStr">
+      <c r="J290" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -18200,7 +18210,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J291" s="13" t="inlineStr">
+      <c r="J291" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -18252,7 +18262,7 @@
           <t>HTTP 200 returned with public fields</t>
         </is>
       </c>
-      <c r="J292" s="13" t="inlineStr">
+      <c r="J292" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -18304,7 +18314,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J293" s="13" t="inlineStr">
+      <c r="J293" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -18356,7 +18366,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J294" s="13" t="inlineStr">
+      <c r="J294" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -18405,10 +18415,10 @@
       </c>
       <c r="I295" s="7" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J295" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J295" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -18457,10 +18467,10 @@
       </c>
       <c r="I296" s="12" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J296" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J296" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -18512,7 +18522,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J297" s="13" t="inlineStr">
+      <c r="J297" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -18564,7 +18574,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J298" s="13" t="inlineStr">
+      <c r="J298" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -18616,7 +18626,7 @@
           <t>HTTP 200 returned with public fields</t>
         </is>
       </c>
-      <c r="J299" s="13" t="inlineStr">
+      <c r="J299" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -18668,7 +18678,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J300" s="13" t="inlineStr">
+      <c r="J300" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -18720,7 +18730,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J301" s="13" t="inlineStr">
+      <c r="J301" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -18769,10 +18779,10 @@
       </c>
       <c r="I302" s="12" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J302" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J302" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -18821,10 +18831,10 @@
       </c>
       <c r="I303" s="7" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J303" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J303" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -18876,7 +18886,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J304" s="13" t="inlineStr">
+      <c r="J304" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -18928,7 +18938,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J305" s="13" t="inlineStr">
+      <c r="J305" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -18980,7 +18990,7 @@
           <t>HTTP 200 returned with public fields</t>
         </is>
       </c>
-      <c r="J306" s="13" t="inlineStr">
+      <c r="J306" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -19032,7 +19042,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J307" s="13" t="inlineStr">
+      <c r="J307" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -19084,7 +19094,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J308" s="13" t="inlineStr">
+      <c r="J308" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -19133,10 +19143,10 @@
       </c>
       <c r="I309" s="7" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J309" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J309" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -19185,10 +19195,10 @@
       </c>
       <c r="I310" s="12" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J310" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J310" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -19240,7 +19250,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J311" s="13" t="inlineStr">
+      <c r="J311" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -19292,7 +19302,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J312" s="13" t="inlineStr">
+      <c r="J312" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -19344,7 +19354,7 @@
           <t>HTTP 401 Authorization token required</t>
         </is>
       </c>
-      <c r="J313" s="13" t="inlineStr">
+      <c r="J313" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -19396,7 +19406,7 @@
           <t>HTTP 401 Invalid token: Signature verification failed</t>
         </is>
       </c>
-      <c r="J314" s="13" t="inlineStr">
+      <c r="J314" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -19448,7 +19458,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J315" s="13" t="inlineStr">
+      <c r="J315" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -19500,7 +19510,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J316" s="13" t="inlineStr">
+      <c r="J316" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -19549,10 +19559,10 @@
       </c>
       <c r="I317" s="7" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J317" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J317" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -19601,10 +19611,10 @@
       </c>
       <c r="I318" s="12" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J318" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J318" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -19656,7 +19666,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J319" s="13" t="inlineStr">
+      <c r="J319" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -19708,7 +19718,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J320" s="13" t="inlineStr">
+      <c r="J320" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -19760,7 +19770,7 @@
           <t>HTTP 401 Authorization token required</t>
         </is>
       </c>
-      <c r="J321" s="13" t="inlineStr">
+      <c r="J321" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -19812,7 +19822,7 @@
           <t>HTTP 401 Invalid token: Signature verification failed</t>
         </is>
       </c>
-      <c r="J322" s="13" t="inlineStr">
+      <c r="J322" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -19864,7 +19874,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J323" s="13" t="inlineStr">
+      <c r="J323" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -19916,7 +19926,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J324" s="13" t="inlineStr">
+      <c r="J324" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -19965,10 +19975,10 @@
       </c>
       <c r="I325" s="7" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J325" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J325" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -20017,10 +20027,10 @@
       </c>
       <c r="I326" s="12" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J326" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J326" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -20072,7 +20082,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J327" s="13" t="inlineStr">
+      <c r="J327" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -20124,7 +20134,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J328" s="13" t="inlineStr">
+      <c r="J328" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -20176,7 +20186,7 @@
           <t>HTTP 401 Authorization token required</t>
         </is>
       </c>
-      <c r="J329" s="13" t="inlineStr">
+      <c r="J329" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -20228,7 +20238,7 @@
           <t>HTTP 401 Invalid token: Signature verification failed</t>
         </is>
       </c>
-      <c r="J330" s="13" t="inlineStr">
+      <c r="J330" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -20280,7 +20290,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J331" s="13" t="inlineStr">
+      <c r="J331" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -20332,7 +20342,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J332" s="13" t="inlineStr">
+      <c r="J332" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -20381,10 +20391,10 @@
       </c>
       <c r="I333" s="7" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J333" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J333" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -20433,10 +20443,10 @@
       </c>
       <c r="I334" s="12" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J334" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J334" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -20488,7 +20498,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J335" s="13" t="inlineStr">
+      <c r="J335" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -20540,7 +20550,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J336" s="13" t="inlineStr">
+      <c r="J336" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -20592,7 +20602,7 @@
           <t>HTTP 401 Authorization token required</t>
         </is>
       </c>
-      <c r="J337" s="13" t="inlineStr">
+      <c r="J337" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -20644,7 +20654,7 @@
           <t>HTTP 401 Invalid token: Signature verification failed</t>
         </is>
       </c>
-      <c r="J338" s="13" t="inlineStr">
+      <c r="J338" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -20696,7 +20706,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J339" s="13" t="inlineStr">
+      <c r="J339" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -20748,7 +20758,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J340" s="13" t="inlineStr">
+      <c r="J340" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -20797,10 +20807,10 @@
       </c>
       <c r="I341" s="7" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J341" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J341" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -20849,10 +20859,10 @@
       </c>
       <c r="I342" s="12" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J342" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J342" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -20904,7 +20914,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J343" s="13" t="inlineStr">
+      <c r="J343" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -20956,7 +20966,7 @@
           <t>HTTP 405 Method Not Allowed</t>
         </is>
       </c>
-      <c r="J344" s="13" t="inlineStr">
+      <c r="J344" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -21008,7 +21018,7 @@
           <t>HTTP 401 Authorization token required</t>
         </is>
       </c>
-      <c r="J345" s="13" t="inlineStr">
+      <c r="J345" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -21060,7 +21070,7 @@
           <t>HTTP 401 Invalid token: Signature verification failed</t>
         </is>
       </c>
-      <c r="J346" s="13" t="inlineStr">
+      <c r="J346" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -21112,7 +21122,7 @@
           <t>Parameter bound safely via SQLAlchemy ORM; no SQL syntax leak</t>
         </is>
       </c>
-      <c r="J347" s="13" t="inlineStr">
+      <c r="J347" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -21164,7 +21174,7 @@
           <t>Returned as inert string in JSON response; safe</t>
         </is>
       </c>
-      <c r="J348" s="13" t="inlineStr">
+      <c r="J348" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -21213,10 +21223,10 @@
       </c>
       <c r="I349" s="7" t="inlineStr">
         <is>
-          <t>All standard security headers populated: X-Content-Type-Options: nosniff, X-Frame-Options: DENY, HSTS, CSP enforced via @app.after_request.</t>
-        </is>
-      </c>
-      <c r="J349" s="13" t="inlineStr">
+          <t>All standard security headers verified (CSP, X-Frame-Options, HSTS, X-Content-Type-Options via @app.after_request)</t>
+        </is>
+      </c>
+      <c r="J349" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -21265,10 +21275,10 @@
       </c>
       <c r="I350" s="12" t="inlineStr">
         <is>
-          <t>Cross-origin requests from unauthorized origins rejected. Access restricted strictly to whitelisted production/dev origins.</t>
-        </is>
-      </c>
-      <c r="J350" s="13" t="inlineStr">
+          <t>CORS origin restricted to authorized whitelist (https://orpha-ai.vercel.app); unauthorized origins rejected</t>
+        </is>
+      </c>
+      <c r="J350" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -21320,7 +21330,7 @@
           <t>Safely validated without server crash or unhandled exception</t>
         </is>
       </c>
-      <c r="J351" s="13" t="inlineStr">
+      <c r="J351" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>

</xml_diff>